<commit_message>
feat: Stabilize login execution flow with robust interpretation, locator handling, and step-level evidence
</commit_message>
<xml_diff>
--- a/docs/TestCases_Login_Module_Sample_V2.xlsx
+++ b/docs/TestCases_Login_Module_Sample_V2.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -442,18 +442,18 @@
         <v>User account exists and user is on home page</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d_
-2. Click Sign In button in header_x000d_
-3. Enter email in Email field_x000d_
-4. Enter password in Password field_x000d_
-5. Click Login button_x000d_
-6. Verify dashboard is visible</v>
+        <v xml:space="preserve">1. Open the website
+2. In the header, click the Sign In link
+3. Enter email in the Email field
+4. Enter password in the Password field
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
+6. Assert text Vishw is visible.</v>
       </c>
       <c r="G2" t="str">
-        <v>email: user@example.com; password: Password123</v>
+        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
       </c>
       <c r="H2" t="str">
-        <v>User should be logged in and redirected to dashboard</v>
+        <v>User is logged in successfully and text Vishw is visible in header account area.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Stabilize Step Interpretation and Locator Resolution for Reliable UI Automation
</commit_message>
<xml_diff>
--- a/docs/TestCases_Login_Module_Sample_V2.xlsx
+++ b/docs/TestCases_Login_Module_Sample_V2.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,23 +442,117 @@
         <v>User account exists and user is on home page</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d_
+2. In the header, click the Sign In link_x000d__x000d__x000d__x000d_
+3. Enter email in the Email field_x000d__x000d__x000d__x000d_
+4. Enter password in the Password field_x000d__x000d__x000d__x000d_
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d_
+6. Assert text Vishw is visible.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
+      </c>
+      <c r="H2" t="str">
+        <v>User is logged in successfully and text Vishw is visible in header account area.</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>Login</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TC_LOGIN_002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Login with wrong email and right password</v>
+      </c>
+      <c r="D3" t="str">
+        <v>User attempts login with invalid email and valid password</v>
+      </c>
+      <c r="E3" t="str">
+        <v>User is on home page; a valid password is available for an existing account format.</v>
+      </c>
+      <c r="F3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d_
+2. In the header, click the Sign In link_x000d__x000d__x000d__x000d_
+3. Enter wrong email in the Email field_x000d__x000d__x000d__x000d_
+4. Enter password in the Password field_x000d__x000d__x000d__x000d_
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d_
+6. Verify popup message Customer account not found is visible.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>email: wrong.user@example.com; password: Password123</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Login fails and an error popup/modal is shown with message Customer account not found.</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>Brands</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TC_BRANDS_001</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Navigate to Brands page from main nav</v>
+      </c>
+      <c r="D4" t="str">
+        <v>User opens Brands page using the top navigation link</v>
+      </c>
+      <c r="E4" t="str">
+        <v>User is on the website home page and main navigation is visible.</v>
+      </c>
+      <c r="F4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website_x000d_
+2. Click Brands link_x000d_
+3. Verify text Trusted Brands is visible</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Brands page opens and Trusted Brands section is visible.</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>Checkout</v>
+      </c>
+      <c r="B5" t="str">
+        <v>TC_CHECKOUT_001</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Login and navigate to checkout from product modal</v>
+      </c>
+      <c r="D5" t="str">
+        <v>User logs in, adds first Lights product to cart, and proceeds to checkout from modal.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Valid user account exists and products are available in Shop &gt; Lights.</v>
+      </c>
+      <c r="F5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open the website
 2. In the header, click the Sign In link
 3. Enter email in the Email field
 4. Enter password in the Password field
 5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
-6. Assert text Vishw is visible.</v>
-      </c>
-      <c r="G2" t="str">
+6. Assert text Vishw is visible.
+7. Hover on Shop
+8. Click Lights
+9. Click Add to Cart link of first product
+10. A modal will appear, click the Checkout Now link</v>
+      </c>
+      <c r="G5" t="str">
         <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
       </c>
-      <c r="H2" t="str">
-        <v>User is logged in successfully and text Vishw is visible in header account area.</v>
+      <c r="H5" t="str">
+        <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Live-safe runs, selector caching, step retries, and interpreter hardening
</commit_message>
<xml_diff>
--- a/docs/TestCases_Login_Module_Sample_V2.xlsx
+++ b/docs/TestCases_Login_Module_Sample_V2.xlsx
@@ -540,8 +540,9 @@
 6. Assert text Vishw is visible.
 7. Hover on Shop
 8. Click Lights
-9. Click Add to Cart link of first product
-10. A modal will appear, click the Checkout Now link</v>
+9. Click first Add to Cart button
+10. Assert modal/dialog with text Checkout Now is visible
+11. Click link Checkout Now</v>
       </c>
       <c r="G5" t="str">
         <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>

</xml_diff>

<commit_message>
feat: Deterministic Ollama outputs + ordinal “Add to cart” locators
</commit_message>
<xml_diff>
--- a/docs/TestCases_Login_Module_Sample_V2.xlsx
+++ b/docs/TestCases_Login_Module_Sample_V2.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -551,9 +551,45 @@
         <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now.</v>
       </c>
     </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>Checkout</v>
+      </c>
+      <c r="B6" t="str">
+        <v>TC_CHECKOUT_002</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Login and navigate to checkout from product modal</v>
+      </c>
+      <c r="D6" t="str">
+        <v>User logs in, adds first Lights product to cart, and proceeds to checkout from modal.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Valid user account exists and products are available in Shop &gt; Lights.</v>
+      </c>
+      <c r="F6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website
+2. In the header, click the Sign In link
+3. Enter email in the Email field
+4. Enter password in the Password field
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
+6. Assert text Vishw is visible.
+7. Hover on Shop
+8. Click Lights
+9. Click second Add to Cart button
+10. Assert modal/dialog with text Checkout Now is visible
+11. Click link Checkout Now</v>
+      </c>
+      <c r="G6" t="str">
+        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
+      </c>
+      <c r="H6" t="str">
+        <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: Improve locator fallback and visible-text assertions for search flows
</commit_message>
<xml_diff>
--- a/docs/TestCases_Login_Module_Sample_V2.xlsx
+++ b/docs/TestCases_Login_Module_Sample_V2.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,11 +442,11 @@
         <v>User account exists and user is on home page</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d_
-2. In the header, click the Sign In link_x000d__x000d__x000d__x000d_
-3. Enter email in the Email field_x000d__x000d__x000d__x000d_
-4. Enter password in the Password field_x000d__x000d__x000d__x000d_
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d__x000d_
+2. In the header, click the Sign In link_x000d__x000d__x000d__x000d__x000d_
+3. Enter email in the Email field_x000d__x000d__x000d__x000d__x000d_
+4. Enter password in the Password field_x000d__x000d__x000d__x000d__x000d_
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d__x000d_
 6. Assert text Vishw is visible.</v>
       </c>
       <c r="G2" t="str">
@@ -473,11 +473,11 @@
         <v>User is on home page; a valid password is available for an existing account format.</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d_
-2. In the header, click the Sign In link_x000d__x000d__x000d__x000d_
-3. Enter wrong email in the Email field_x000d__x000d__x000d__x000d_
-4. Enter password in the Password field_x000d__x000d__x000d__x000d_
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d__x000d_
+2. In the header, click the Sign In link_x000d__x000d__x000d__x000d__x000d_
+3. Enter wrong email in the Email field_x000d__x000d__x000d__x000d__x000d_
+4. Enter password in the Password field_x000d__x000d__x000d__x000d__x000d_
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d__x000d_
 6. Verify popup message Customer account not found is visible.</v>
       </c>
       <c r="G3" t="str">
@@ -504,12 +504,9 @@
         <v>User is on the website home page and main navigation is visible.</v>
       </c>
       <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d_
-2. Click Brands link_x000d_
+        <v xml:space="preserve">1. Open the website_x000d__x000d_
+2. Click Brands link_x000d__x000d_
 3. Verify text Trusted Brands is visible</v>
-      </c>
-      <c r="G4" t="str">
-        <v/>
       </c>
       <c r="H4" t="str">
         <v>Brands page opens and Trusted Brands section is visible.</v>
@@ -532,16 +529,16 @@
         <v>Valid user account exists and products are available in Shop &gt; Lights.</v>
       </c>
       <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website
-2. In the header, click the Sign In link
-3. Enter email in the Email field
-4. Enter password in the Password field
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
-6. Assert text Vishw is visible.
-7. Hover on Shop
-8. Click Lights
-9. Click first Add to Cart button
-10. Assert modal/dialog with text Checkout Now is visible
+        <v xml:space="preserve">1. Open the website_x000d_
+2. In the header, click the Sign In link_x000d_
+3. Enter email in the Email field_x000d_
+4. Enter password in the Password field_x000d_
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d_
+6. Assert text Vishw is visible._x000d_
+7. Hover on Shop_x000d_
+8. Click Lights_x000d_
+9. Click first Add to Cart button_x000d_
+10. Assert modal/dialog with text Checkout Now is visible_x000d_
 11. Click link Checkout Now</v>
       </c>
       <c r="G5" t="str">
@@ -568,16 +565,16 @@
         <v>Valid user account exists and products are available in Shop &gt; Lights.</v>
       </c>
       <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website
-2. In the header, click the Sign In link
-3. Enter email in the Email field
-4. Enter password in the Password field
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
-6. Assert text Vishw is visible.
-7. Hover on Shop
-8. Click Lights
-9. Click second Add to Cart button
-10. Assert modal/dialog with text Checkout Now is visible
+        <v xml:space="preserve">1. Open the website_x000d_
+2. In the header, click the Sign In link_x000d_
+3. Enter email in the Email field_x000d_
+4. Enter password in the Password field_x000d_
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d_
+6. Assert text Vishw is visible._x000d_
+7. Hover on Shop_x000d_
+8. Click Lights_x000d_
+9. Click second Add to Cart button_x000d_
+10. Assert modal/dialog with text Checkout Now is visible_x000d_
 11. Click link Checkout Now</v>
       </c>
       <c r="G6" t="str">
@@ -585,11 +582,40 @@
       </c>
       <c r="H6" t="str">
         <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now.</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>Search</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TC_SEARCH_001</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Verify search functionality with valid keyword</v>
+      </c>
+      <c r="D7" t="str">
+        <v>User searches for 'sleipner' from website search bar</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Website is up and accessible; search input and Search button are visible and enabled</v>
+      </c>
+      <c r="F7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website
+2. Enter 'sleipner' in the search field
+3. Click on the Search button
+4. Assert text Sleipner is visible.</v>
+      </c>
+      <c r="G7" t="str">
+        <v>search_keyword=sleipner</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Search results are displayed and text sleipner is visible</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Added scroll action, staged viewport nudge, and always scroll before interactions
</commit_message>
<xml_diff>
--- a/docs/TestCases_Login_Module_Sample_V2.xlsx
+++ b/docs/TestCases_Login_Module_Sample_V2.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:U42"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,195 +427,565 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>Login</v>
+        <v>Footer</v>
       </c>
       <c r="B2" t="str">
-        <v>TC_LOGIN_001</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Valid login with registered user</v>
+        <v>Navigate to About Imtra page from footer</v>
       </c>
       <c r="D2" t="str">
-        <v>User logs in successfully with valid credentials</v>
+        <v>User opens the About Imtra page using the footer Pages link</v>
       </c>
       <c r="E2" t="str">
-        <v>User account exists and user is on home page</v>
+        <v>Website is up and accessible, and footer links are visible</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d__x000d_
-2. In the header, click the Sign In link_x000d__x000d__x000d__x000d__x000d_
-3. Enter email in the Email field_x000d__x000d__x000d__x000d__x000d_
-4. Enter password in the Password field_x000d__x000d__x000d__x000d__x000d_
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d__x000d_
-6. Assert text Vishw is visible.</v>
-      </c>
-      <c r="G2" t="str">
-        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
+        <v xml:space="preserve">1. Open the website
+2. Scroll to the footer section
+3. In the Footer, Click the Careers link
+4. Verify text Careers is visible</v>
       </c>
       <c r="H2" t="str">
-        <v>User is logged in successfully and text Vishw is visible in header account area.</v>
+        <v>About Imtra page opens successfully and page title About Imtra - IMTRA is visible.</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>Login</v>
+        <v>Footer</v>
       </c>
       <c r="B3" t="str">
-        <v>TC_LOGIN_002</v>
+        <v>TC_FOOTER_001</v>
       </c>
       <c r="C3" t="str">
-        <v>Login with wrong email and right password</v>
+        <v>Navigate to About Imtra page from footer</v>
       </c>
       <c r="D3" t="str">
-        <v>User attempts login with invalid email and valid password</v>
+        <v>User opens the About Imtra page using the footer Pages link</v>
       </c>
       <c r="E3" t="str">
-        <v>User is on home page; a valid password is available for an existing account format.</v>
+        <v>Website is up and accessible, and footer links are visible</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d__x000d__x000d__x000d__x000d_
-2. In the header, click the Sign In link_x000d__x000d__x000d__x000d__x000d_
-3. Enter wrong email in the Email field_x000d__x000d__x000d__x000d__x000d_
-4. Enter password in the Password field_x000d__x000d__x000d__x000d__x000d_
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d__x000d__x000d__x000d__x000d_
-6. Verify popup message Customer account not found is visible.</v>
-      </c>
-      <c r="G3" t="str">
-        <v>email: wrong.user@example.com; password: Password123</v>
+        <v xml:space="preserve">1. Open the website
+2. Scroll to the footer section
+3. In the Footer, Click the About IMTRA link
+4. Verify text About IMTRA is visible</v>
       </c>
       <c r="H3" t="str">
-        <v>Login fails and an error popup/modal is shown with message Customer account not found.</v>
+        <v>About Imtra page opens successfully and page title About Imtra - IMTRA is visible.</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>Brands</v>
+        <v>My Account User Login</v>
       </c>
       <c r="B4" t="str">
-        <v>TC_BRANDS_001</v>
+        <v>TC_USER_LOGIN_001</v>
       </c>
       <c r="C4" t="str">
-        <v>Navigate to Brands page from main nav</v>
+        <v>Search Existing User By Partial Name</v>
       </c>
       <c r="D4" t="str">
-        <v>User opens Brands page using the top navigation link</v>
+        <v>User searches by Firstname in searchbar</v>
       </c>
       <c r="E4" t="str">
-        <v>User is on the website home page and main navigation is visible.</v>
+        <v>User is logged in and users data are visible on the user login page and search input are visible and enabled_x000d_</v>
       </c>
       <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d__x000d_
-2. Click Brands link_x000d__x000d_
-3. Verify text Trusted Brands is visible</v>
+        <v xml:space="preserve">1. Open the website.
+2. In the header section, click the Sign In link.
+3. Enter a valid email address in the Email field.
+4. Enter a valid password in the Password field.
+5. Click the SIGN IN button (primary full-width submit button).
+6. Verify that the text Nikhil is visible on the page.
+7. Hover on Nikhil.
+8. Click on Company Settings link.
+9. Click on User Login link.
+10. Enter the search keyword into the Search users field.
+11. Verify text Nikhil Shimpi is visible</v>
+      </c>
+      <c r="G4" t="str">
+        <v>email: nikhils@redefinesolutions.com; password: Admin@1234; search_keyword=Nikhil</v>
       </c>
       <c r="H4" t="str">
-        <v>Brands page opens and Trusted Brands section is visible.</v>
+        <v>Search results are displayed and text nikhil is visible_x000d_</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>Checkout</v>
+        <v>Login</v>
       </c>
       <c r="B5" t="str">
-        <v>TC_CHECKOUT_001</v>
+        <v>TC_LOGIN_001</v>
       </c>
       <c r="C5" t="str">
-        <v>Login and navigate to checkout from product modal</v>
+        <v>Valid login with registered user</v>
       </c>
       <c r="D5" t="str">
-        <v>User logs in, adds first Lights product to cart, and proceeds to checkout from modal.</v>
+        <v>User logs in successfully with valid credentials</v>
       </c>
       <c r="E5" t="str">
-        <v>Valid user account exists and products are available in Shop &gt; Lights.</v>
+        <v>User account exists and user is on home page_x000d_</v>
       </c>
       <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d_
-2. In the header, click the Sign In link_x000d_
-3. Enter email in the Email field_x000d_
-4. Enter password in the Password field_x000d_
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d_
-6. Assert text Vishw is visible._x000d_
-7. Hover on Shop_x000d_
-8. Click Lights_x000d_
-9. Click first Add to Cart button_x000d_
-10. Assert modal/dialog with text Checkout Now is visible_x000d_
-11. Click link Checkout Now</v>
+        <v xml:space="preserve">1. Open the website
+2. In the header, click the Sign In link
+3. Enter email in the Email field
+4. Enter password in the Password field
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
+6. Verify text Vishw is visible.</v>
       </c>
       <c r="G5" t="str">
         <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
       </c>
       <c r="H5" t="str">
-        <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now.</v>
+        <v>User is logged in successfully and text Vishw is visible in header account area._x000d_</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>Checkout</v>
+        <v>Brands</v>
       </c>
       <c r="B6" t="str">
-        <v>TC_CHECKOUT_002</v>
+        <v>TC_BRANDS_001</v>
       </c>
       <c r="C6" t="str">
-        <v>Login and navigate to checkout from product modal</v>
+        <v>Navigate to Brands page from main nav</v>
       </c>
       <c r="D6" t="str">
-        <v>User logs in, adds first Lights product to cart, and proceeds to checkout from modal.</v>
+        <v>User opens Brands page using the top navigation link</v>
       </c>
       <c r="E6" t="str">
-        <v>Valid user account exists and products are available in Shop &gt; Lights.</v>
+        <v>User is on the website home page and main navigation is visible._x000d_</v>
       </c>
       <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the website_x000d_
-2. In the header, click the Sign In link_x000d_
-3. Enter email in the Email field_x000d_
-4. Enter password in the Password field_x000d_
-5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)_x000d_
-6. Assert text Vishw is visible._x000d_
-7. Hover on Shop_x000d_
-8. Click Lights_x000d_
-9. Click second Add to Cart button_x000d_
-10. Assert modal/dialog with text Checkout Now is visible_x000d_
-11. Click link Checkout Now</v>
+        <v xml:space="preserve">1. Open the website
+2. Click Brands link
+3. Verify text Trusted Brands is visible</v>
       </c>
       <c r="G6" t="str">
-        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now.</v>
+        <v>Brands page opens and Trusted Brands section is visible._x000d_</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
+        <v>Checkout</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TC_CHECKOUT_001</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Login and navigate to checkout from product modal</v>
+      </c>
+      <c r="D7" t="str">
+        <v>User logs in, adds first Lights product to cart, and proceeds to checkout from modal.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Valid user account exists and products are available in Shop &gt; Lights._x000d_</v>
+      </c>
+      <c r="F7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website
+2. In the header, click the Sign In link
+3. Enter email in the Email field
+4. Enter password in the Password field
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
+6. Verify text Vishw is visible.
+7. Hover on Shop
+8. Click Lights
+9. Click first Add to Cart button
+10. Assert modal/dialog with text Checkout Now is visible
+11. Click link Checkout Now</v>
+      </c>
+      <c r="G7" t="str">
+        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
+      </c>
+      <c r="H7" t="str">
+        <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now._x000d_</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>Checkout</v>
+      </c>
+      <c r="B8" t="str">
+        <v>TC_CHECKOUT_002</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Login and navigate to checkout from product modal</v>
+      </c>
+      <c r="D8" t="str">
+        <v>User logs in, adds first Lights product to cart, and proceeds to checkout from modal.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Valid user account exists and products are available in Shop &gt; Lights._x000d_</v>
+      </c>
+      <c r="F8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the website
+2. In the header, click the Sign In link
+3. Enter email in the Email field
+4. Enter password in the Password field
+5. On the login form, click the SIGN IN submit button (primary full-width button, type submit)
+6. Verify text Vishw is visible.
+7. Hover on Shop
+8. Click Lights
+9. Click second Add to Cart button
+10. Assert modal/dialog with text Checkout Now is visible
+11. Click link Checkout Now</v>
+      </c>
+      <c r="G8" t="str">
+        <v>email: vishw@redefinesolutions.com; password: Vishw@123</v>
+      </c>
+      <c r="H8" t="str">
+        <v>User reaches checkout flow after adding first product from Lights and clicking Checkout Now._x000d_</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
         <v>Search</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B9" t="str">
         <v>TC_SEARCH_001</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C9" t="str">
         <v>Verify search functionality with valid keyword</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D9" t="str">
         <v>User searches for 'sleipner' from website search bar</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E9" t="str">
         <v>Website is up and accessible; search input and Search button are visible and enabled</v>
       </c>
-      <c r="F7" t="str" xml:space="preserve">
+      <c r="F9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open the website
 2. Enter 'sleipner' in the search field
 3. Click on the Search button
-4. Assert text Sleipner is visible.</v>
-      </c>
-      <c r="G7" t="str">
+4. Verify text Sleipner is visible.</v>
+      </c>
+      <c r="G9" t="str">
         <v>search_keyword=sleipner</v>
       </c>
-      <c r="H7" t="str">
+      <c r="H9" t="str">
         <v>Search results are displayed and text sleipner is visible</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v/>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v/>
+      </c>
+      <c r="N42" t="str">
+        <v/>
+      </c>
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U42"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>